<commit_message>
criação de um menu para acessar opções do mercado interno, consulta, edição de recebimento e cancelamento de contrato
</commit_message>
<xml_diff>
--- a/db/OLEO26RC.xlsx
+++ b/db/OLEO26RC.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1238" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1251" uniqueCount="403">
   <si>
     <t>DATA</t>
   </si>
@@ -692,6 +692,9 @@
   </si>
   <si>
     <t>20392</t>
+  </si>
+  <si>
+    <t>25.00</t>
   </si>
   <si>
     <t>074</t>
@@ -1577,7 +1580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O192"/>
+  <dimension ref="A1:O193"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.77734375" customWidth="1"/>
@@ -4826,8 +4829,8 @@
       <c r="G81" s="2">
         <v>17090.13</v>
       </c>
-      <c r="H81" s="2">
-        <v>16833.78</v>
+      <c r="H81" s="2" t="s">
+        <v>225</v>
       </c>
       <c r="I81" s="2">
         <v>0</v>
@@ -4856,7 +4859,7 @@
         <v>27</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D82" s="1" t="s">
         <v>17</v>
@@ -4874,10 +4877,10 @@
         <v>0</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K82" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="L82" s="1" t="s">
         <v>19</v>
@@ -4897,7 +4900,7 @@
         <v>27</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D83" s="1" t="s">
         <v>17</v>
@@ -4915,10 +4918,10 @@
         <v>0</v>
       </c>
       <c r="J83" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K83" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L83" s="1" t="s">
         <v>19</v>
@@ -4938,13 +4941,13 @@
         <v>27</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D84" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G84" s="2">
         <v>28793.43</v>
@@ -4956,10 +4959,10 @@
         <v>0</v>
       </c>
       <c r="J84" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K84" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L84" s="1" t="s">
         <v>19</v>
@@ -4979,7 +4982,7 @@
         <v>27</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D85" s="1" t="s">
         <v>17</v>
@@ -5020,7 +5023,7 @@
         <v>27</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>17</v>
@@ -5038,10 +5041,10 @@
         <v>0</v>
       </c>
       <c r="J86" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K86" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L86" s="1" t="s">
         <v>19</v>
@@ -5061,7 +5064,7 @@
         <v>27</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D87" s="1" t="s">
         <v>17</v>
@@ -5079,10 +5082,10 @@
         <v>0</v>
       </c>
       <c r="J87" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K87" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="L87" s="1" t="s">
         <v>19</v>
@@ -5102,7 +5105,7 @@
         <v>27</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>17</v>
@@ -5120,10 +5123,10 @@
         <v>0</v>
       </c>
       <c r="J88" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K88" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="L88" s="1" t="s">
         <v>19</v>
@@ -5164,7 +5167,7 @@
         <v>19</v>
       </c>
       <c r="K89" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L89" s="1" t="s">
         <v>19</v>
@@ -5184,7 +5187,7 @@
         <v>27</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D90" s="1" t="s">
         <v>17</v>
@@ -5202,10 +5205,10 @@
         <v>0</v>
       </c>
       <c r="J90" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K90" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="L90" s="1" t="s">
         <v>19</v>
@@ -5225,7 +5228,7 @@
         <v>27</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D91" s="1" t="s">
         <v>17</v>
@@ -5243,10 +5246,10 @@
         <v>0</v>
       </c>
       <c r="J91" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K91" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="L91" s="1" t="s">
         <v>19</v>
@@ -5307,13 +5310,13 @@
         <v>27</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D93" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G93" s="2">
         <v>28252.81</v>
@@ -5325,10 +5328,10 @@
         <v>0</v>
       </c>
       <c r="J93" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="K93" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L93" s="1" t="s">
         <v>19</v>
@@ -5348,13 +5351,13 @@
         <v>27</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D94" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G94" s="2">
         <v>16842.24</v>
@@ -5366,10 +5369,10 @@
         <v>0</v>
       </c>
       <c r="J94" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K94" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L94" s="1" t="s">
         <v>19</v>
@@ -5389,7 +5392,7 @@
         <v>27</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D95" s="1" t="s">
         <v>17</v>
@@ -5407,10 +5410,10 @@
         <v>0</v>
       </c>
       <c r="J95" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K95" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="L95" s="1" t="s">
         <v>19</v>
@@ -5430,7 +5433,7 @@
         <v>27</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D96" s="1" t="s">
         <v>17</v>
@@ -5448,10 +5451,10 @@
         <v>0</v>
       </c>
       <c r="J96" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K96" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="L96" s="1" t="s">
         <v>19</v>
@@ -5471,7 +5474,7 @@
         <v>85</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D97" s="1" t="s">
         <v>17</v>
@@ -5489,10 +5492,10 @@
         <v>0</v>
       </c>
       <c r="J97" s="1" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="K97" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="L97" s="1" t="s">
         <v>19</v>
@@ -5512,13 +5515,13 @@
         <v>27</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D98" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G98" s="2">
         <v>5584.86</v>
@@ -5530,10 +5533,10 @@
         <v>0</v>
       </c>
       <c r="J98" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K98" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L98" s="1" t="s">
         <v>19</v>
@@ -5553,13 +5556,13 @@
         <v>27</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D99" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G99" s="2">
         <v>1347.92</v>
@@ -5571,10 +5574,10 @@
         <v>0</v>
       </c>
       <c r="J99" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K99" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L99" s="1" t="s">
         <v>19</v>
@@ -5594,7 +5597,7 @@
         <v>27</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D100" s="1" t="s">
         <v>17</v>
@@ -5612,10 +5615,10 @@
         <v>0</v>
       </c>
       <c r="J100" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K100" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="L100" s="1" t="s">
         <v>19</v>
@@ -5635,7 +5638,7 @@
         <v>27</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D101" s="1" t="s">
         <v>17</v>
@@ -5653,10 +5656,10 @@
         <v>0</v>
       </c>
       <c r="J101" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K101" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L101" s="1" t="s">
         <v>19</v>
@@ -5697,7 +5700,7 @@
         <v>19</v>
       </c>
       <c r="K102" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L102" s="1" t="s">
         <v>19</v>
@@ -5779,7 +5782,7 @@
         <v>19</v>
       </c>
       <c r="K104" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="L104" s="1" t="s">
         <v>19</v>
@@ -5799,7 +5802,7 @@
         <v>27</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D105" s="1" t="s">
         <v>17</v>
@@ -5817,10 +5820,10 @@
         <v>0</v>
       </c>
       <c r="J105" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K105" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L105" s="1" t="s">
         <v>19</v>
@@ -5840,13 +5843,13 @@
         <v>27</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D106" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G106" s="2">
         <v>1046.36</v>
@@ -5858,10 +5861,10 @@
         <v>0</v>
       </c>
       <c r="J106" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="K106" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="L106" s="1" t="s">
         <v>19</v>
@@ -5881,7 +5884,7 @@
         <v>27</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D107" s="1" t="s">
         <v>17</v>
@@ -5899,10 +5902,10 @@
         <v>0</v>
       </c>
       <c r="J107" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K107" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="L107" s="1" t="s">
         <v>19</v>
@@ -5922,7 +5925,7 @@
         <v>27</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D108" s="1" t="s">
         <v>17</v>
@@ -5940,10 +5943,10 @@
         <v>0</v>
       </c>
       <c r="J108" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="K108" s="1" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="L108" s="1" t="s">
         <v>19</v>
@@ -5963,13 +5966,13 @@
         <v>27</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D109" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G109" s="2">
         <v>2237.12</v>
@@ -5981,10 +5984,10 @@
         <v>0</v>
       </c>
       <c r="J109" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="K109" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="L109" s="1" t="s">
         <v>19</v>
@@ -6209,13 +6212,13 @@
         <v>27</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D115" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F115" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G115" s="2">
         <v>15000</v>
@@ -6227,10 +6230,10 @@
         <v>0</v>
       </c>
       <c r="J115" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="K115" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L115" s="1" t="s">
         <v>19</v>
@@ -6250,13 +6253,13 @@
         <v>27</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D116" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F116" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G116" s="2">
         <v>2268.66</v>
@@ -6268,10 +6271,10 @@
         <v>0</v>
       </c>
       <c r="J116" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="K116" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="L116" s="1" t="s">
         <v>19</v>
@@ -6291,13 +6294,13 @@
         <v>27</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D117" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F117" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G117" s="2">
         <v>15638.04</v>
@@ -6309,10 +6312,10 @@
         <v>0</v>
       </c>
       <c r="J117" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="K117" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L117" s="1" t="s">
         <v>19</v>
@@ -6332,13 +6335,13 @@
         <v>27</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D118" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F118" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G118" s="2">
         <v>2324.44</v>
@@ -6350,10 +6353,10 @@
         <v>0</v>
       </c>
       <c r="J118" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="K118" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L118" s="1" t="s">
         <v>19</v>
@@ -6373,7 +6376,7 @@
         <v>27</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D119" s="1" t="s">
         <v>17</v>
@@ -6391,10 +6394,10 @@
         <v>0</v>
       </c>
       <c r="J119" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K119" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L119" s="1" t="s">
         <v>19</v>
@@ -6414,7 +6417,7 @@
         <v>27</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D120" s="1" t="s">
         <v>17</v>
@@ -6431,13 +6434,13 @@
         <v>27</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D121" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F121" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="122" spans="1:14" x14ac:dyDescent="0.25">
@@ -6448,7 +6451,7 @@
         <v>27</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D122" s="1" t="s">
         <v>17</v>
@@ -6466,10 +6469,10 @@
         <v>0</v>
       </c>
       <c r="J122" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="K122" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L122" s="1" t="s">
         <v>19</v>
@@ -6489,7 +6492,7 @@
         <v>15</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D123" s="1" t="s">
         <v>17</v>
@@ -6507,10 +6510,10 @@
         <v>0</v>
       </c>
       <c r="J123" s="1" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="K123" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="L123" s="1" t="s">
         <v>19</v>
@@ -6530,7 +6533,7 @@
         <v>27</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D124" s="1" t="s">
         <v>17</v>
@@ -6548,10 +6551,10 @@
         <v>0</v>
       </c>
       <c r="J124" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="K124" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="L124" s="1" t="s">
         <v>19</v>
@@ -6571,13 +6574,13 @@
         <v>27</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D125" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F125" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G125" s="2">
         <v>0</v>
@@ -6600,13 +6603,13 @@
         <v>27</v>
       </c>
       <c r="C126" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F126" s="1" t="s">
         <v>308</v>
-      </c>
-      <c r="D126" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="F126" s="1" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="127" spans="1:14" x14ac:dyDescent="0.25">
@@ -6617,7 +6620,7 @@
         <v>85</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D127" s="1" t="s">
         <v>17</v>
@@ -6635,10 +6638,10 @@
         <v>0</v>
       </c>
       <c r="J127" s="1" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="K127" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="L127" s="1" t="s">
         <v>19</v>
@@ -6655,7 +6658,7 @@
         <v>15</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D128" s="1" t="s">
         <v>17</v>
@@ -6672,7 +6675,7 @@
         <v>27</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D129" s="1" t="s">
         <v>17</v>
@@ -6689,13 +6692,13 @@
         <v>27</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D130" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F130" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
@@ -6706,13 +6709,13 @@
         <v>27</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D131" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F131" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="132" spans="1:14" x14ac:dyDescent="0.25">
@@ -6723,7 +6726,7 @@
         <v>27</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D132" s="1" t="s">
         <v>17</v>
@@ -6741,10 +6744,10 @@
         <v>0</v>
       </c>
       <c r="J132" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K132" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="L132" s="1" t="s">
         <v>19</v>
@@ -6764,7 +6767,7 @@
         <v>15</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D133" s="1" t="s">
         <v>17</v>
@@ -6781,13 +6784,13 @@
         <v>27</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D134" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G134" s="2">
         <v>0</v>
@@ -6813,7 +6816,7 @@
         <v>27</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D135" s="1" t="s">
         <v>17</v>
@@ -6831,10 +6834,10 @@
         <v>0</v>
       </c>
       <c r="J135" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K135" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="N135" s="2">
         <v>922.74</v>
@@ -6866,10 +6869,10 @@
         <v>0</v>
       </c>
       <c r="J136" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K136" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L136" s="1" t="s">
         <v>19</v>
@@ -6907,10 +6910,10 @@
         <v>0</v>
       </c>
       <c r="J137" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K137" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L137" s="1" t="s">
         <v>19</v>
@@ -6948,10 +6951,10 @@
         <v>0</v>
       </c>
       <c r="J138" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K138" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L138" s="1" t="s">
         <v>19</v>
@@ -6989,10 +6992,10 @@
         <v>0</v>
       </c>
       <c r="J139" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K139" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L139" s="1" t="s">
         <v>19</v>
@@ -7003,6 +7006,10 @@
       <c r="N139" s="2">
         <v>1578.21</v>
       </c>
+    </row>
+    <row r="140" spans="3:4" x14ac:dyDescent="0.25">
+      <c r="C140" s="1"/>
+      <c r="D140" s="1"/>
     </row>
     <row r="141" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A141" s="3">
@@ -7012,7 +7019,7 @@
         <v>27</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D141" s="1" t="s">
         <v>17</v>
@@ -7030,10 +7037,10 @@
         <v>0</v>
       </c>
       <c r="J141" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K141" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="L141" s="1" t="s">
         <v>19</v>
@@ -7053,7 +7060,7 @@
         <v>27</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D142" s="1" t="s">
         <v>17</v>
@@ -7071,10 +7078,10 @@
         <v>0</v>
       </c>
       <c r="J142" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="K142" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="N142" s="2">
         <v>1395.06</v>
@@ -7085,16 +7092,16 @@
         <v>46254</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="D143" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F143" s="1" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G143" s="2">
         <v>9610.49</v>
@@ -7106,10 +7113,10 @@
         <v>0</v>
       </c>
       <c r="J143" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K143" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="N143" s="2">
         <v>8355.33</v>
@@ -7123,7 +7130,7 @@
         <v>27</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D144" s="1" t="s">
         <v>17</v>
@@ -7141,10 +7148,10 @@
         <v>0</v>
       </c>
       <c r="J144" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K144" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="L144" s="1" t="s">
         <v>19</v>
@@ -7164,7 +7171,7 @@
         <v>27</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D145" s="1" t="s">
         <v>17</v>
@@ -7181,13 +7188,13 @@
         <v>27</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D146" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F146" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G146" s="2">
         <v>30500</v>
@@ -7199,10 +7206,10 @@
         <v>0</v>
       </c>
       <c r="J146" s="1" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="K146" s="1" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="L146" s="1" t="s">
         <v>19</v>
@@ -7222,7 +7229,7 @@
         <v>27</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D147" s="1" t="s">
         <v>17</v>
@@ -7240,10 +7247,10 @@
         <v>0</v>
       </c>
       <c r="J147" s="1" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K147" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="L147" s="1" t="s">
         <v>19</v>
@@ -7263,13 +7270,13 @@
         <v>27</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="D148" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F148" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G148" s="2">
         <v>15250</v>
@@ -7281,10 +7288,10 @@
         <v>0</v>
       </c>
       <c r="J148" s="1" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K148" s="1" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="L148" s="1" t="s">
         <v>19</v>
@@ -7304,7 +7311,7 @@
         <v>15</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D149" s="1" t="s">
         <v>17</v>
@@ -7321,7 +7328,7 @@
         <v>15</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D150" s="1" t="s">
         <v>17</v>
@@ -7338,13 +7345,13 @@
         <v>27</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D151" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F151" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G151" s="2">
         <v>1142.75</v>
@@ -7356,10 +7363,10 @@
         <v>0</v>
       </c>
       <c r="J151" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K151" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L151" s="1" t="s">
         <v>19</v>
@@ -7379,13 +7386,13 @@
         <v>27</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="D152" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F152" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G152" s="2">
         <v>15750</v>
@@ -7397,10 +7404,10 @@
         <v>0</v>
       </c>
       <c r="J152" s="1" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="K152" s="1" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="L152" s="1" t="s">
         <v>19</v>
@@ -7420,13 +7427,13 @@
         <v>27</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D153" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F153" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G153" s="2">
         <v>15750</v>
@@ -7438,10 +7445,10 @@
         <v>0</v>
       </c>
       <c r="J153" s="1" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="K153" s="1" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="L153" s="1" t="s">
         <v>19</v>
@@ -7458,13 +7465,13 @@
         <v>27</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D154" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F154" s="1" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G154" s="2">
         <v>10084.2</v>
@@ -7476,10 +7483,10 @@
         <v>0</v>
       </c>
       <c r="J154" s="1" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="K154" s="1" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="L154" s="1" t="s">
         <v>19</v>
@@ -7496,7 +7503,7 @@
         <v>85</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D155" s="1" t="s">
         <v>17</v>
@@ -7513,13 +7520,13 @@
         <v>27</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D156" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F156" s="1" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G156" s="2">
         <v>5262.51</v>
@@ -7531,10 +7538,10 @@
         <v>0</v>
       </c>
       <c r="J156" s="1" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="K156" s="1" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="L156" s="1" t="s">
         <v>19</v>
@@ -7551,16 +7558,16 @@
         <v>46267</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D157" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F157" s="1" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G157" s="2">
         <v>7539.44</v>
@@ -7572,10 +7579,10 @@
         <v>0</v>
       </c>
       <c r="J157" s="1" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="K157" s="1" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="N157" s="2">
         <v>6554.77</v>
@@ -7589,13 +7596,13 @@
         <v>27</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D158" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F158" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="159" spans="1:14" x14ac:dyDescent="0.25">
@@ -7606,13 +7613,13 @@
         <v>27</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D159" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F159" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G159" s="2">
         <v>1153.29</v>
@@ -7624,10 +7631,10 @@
         <v>0</v>
       </c>
       <c r="J159" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K159" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L159" s="1" t="s">
         <v>19</v>
@@ -7644,16 +7651,16 @@
         <v>46275</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D160" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F160" s="1" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.25">
@@ -7664,13 +7671,13 @@
         <v>27</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D161" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F161" s="1" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.25">
@@ -7681,7 +7688,7 @@
         <v>27</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D162" s="1" t="s">
         <v>17</v>
@@ -7695,16 +7702,16 @@
         <v>46279</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D163" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F163" s="1" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.25">
@@ -7715,7 +7722,7 @@
         <v>15</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="D164" s="1" t="s">
         <v>17</v>
@@ -7732,7 +7739,7 @@
         <v>15</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D165" s="1" t="s">
         <v>17</v>
@@ -7749,13 +7756,13 @@
         <v>27</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D166" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F166" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G166" s="2">
         <v>0</v>
@@ -7796,10 +7803,10 @@
         <v>0</v>
       </c>
       <c r="J167" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K167" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L167" s="1" t="s">
         <v>19</v>
@@ -7819,13 +7826,13 @@
         <v>27</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D168" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F168" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G168" s="2">
         <v>157.76</v>
@@ -7837,10 +7844,10 @@
         <v>0</v>
       </c>
       <c r="J168" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K168" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L168" s="1" t="s">
         <v>19</v>
@@ -7860,13 +7867,13 @@
         <v>27</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D169" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F169" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G169" s="2">
         <v>11499.2</v>
@@ -7878,10 +7885,10 @@
         <v>0</v>
       </c>
       <c r="J169" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K169" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L169" s="1" t="s">
         <v>19</v>
@@ -7901,7 +7908,7 @@
         <v>27</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D170" s="1" t="s">
         <v>17</v>
@@ -7918,13 +7925,13 @@
         <v>27</v>
       </c>
       <c r="C171" s="1" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D171" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F171" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G171" s="2">
         <v>2374.96</v>
@@ -7936,10 +7943,10 @@
         <v>0</v>
       </c>
       <c r="J171" s="1" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K171" s="1" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L171" s="1" t="s">
         <v>19</v>
@@ -7959,13 +7966,13 @@
         <v>27</v>
       </c>
       <c r="C172" s="1" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D172" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F172" s="1" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G172" s="2">
         <v>0</v>
@@ -7988,7 +7995,7 @@
         <v>15</v>
       </c>
       <c r="C173" s="1" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D173" s="1" t="s">
         <v>17</v>
@@ -8005,7 +8012,7 @@
         <v>27</v>
       </c>
       <c r="C174" s="1" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D174" s="1" t="s">
         <v>17</v>
@@ -8022,7 +8029,7 @@
         <v>27</v>
       </c>
       <c r="C175" s="1" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="D175" s="1" t="s">
         <v>17</v>
@@ -8039,7 +8046,7 @@
         <v>27</v>
       </c>
       <c r="C176" s="1" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D176" s="1" t="s">
         <v>17</v>
@@ -8056,13 +8063,13 @@
         <v>27</v>
       </c>
       <c r="C177" s="1" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D177" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F177" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.25">
@@ -8073,7 +8080,7 @@
         <v>15</v>
       </c>
       <c r="C178" s="1" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D178" s="1" t="s">
         <v>17</v>
@@ -8090,7 +8097,7 @@
         <v>85</v>
       </c>
       <c r="C179" s="1" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="D179" s="1" t="s">
         <v>17</v>
@@ -8107,13 +8114,13 @@
         <v>27</v>
       </c>
       <c r="C180" s="1" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="D180" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F180" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G180" s="2">
         <v>0</v>
@@ -8136,13 +8143,13 @@
         <v>27</v>
       </c>
       <c r="C181" s="1" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D181" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F181" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.25">
@@ -8153,13 +8160,13 @@
         <v>15</v>
       </c>
       <c r="C182" s="1" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D182" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F182" s="1" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.25">
@@ -8170,13 +8177,13 @@
         <v>27</v>
       </c>
       <c r="C183" s="1" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D183" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F183" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="184" spans="1:14" x14ac:dyDescent="0.25">
@@ -8205,10 +8212,10 @@
         <v>0</v>
       </c>
       <c r="J184" s="1" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K184" s="1" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="L184" s="1" t="s">
         <v>19</v>
@@ -8246,10 +8253,10 @@
         <v>0</v>
       </c>
       <c r="J185" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K185" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="L185" s="1" t="s">
         <v>19</v>
@@ -8269,13 +8276,13 @@
         <v>27</v>
       </c>
       <c r="C186" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D186" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F186" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G186" s="2">
         <v>165.95</v>
@@ -8287,10 +8294,10 @@
         <v>0</v>
       </c>
       <c r="J186" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K186" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="L186" s="1" t="s">
         <v>19</v>
@@ -8310,13 +8317,13 @@
         <v>27</v>
       </c>
       <c r="C187" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D187" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F187" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G187" s="2">
         <v>15710.96</v>
@@ -8328,10 +8335,10 @@
         <v>0</v>
       </c>
       <c r="J187" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="K187" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="L187" s="1" t="s">
         <v>19</v>
@@ -8351,13 +8358,13 @@
         <v>27</v>
       </c>
       <c r="C188" s="1" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="D188" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F188" s="1" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.25">
@@ -8368,7 +8375,7 @@
         <v>15</v>
       </c>
       <c r="C189" s="1" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D189" s="1" t="s">
         <v>17</v>
@@ -8394,33 +8401,33 @@
         <v>18</v>
       </c>
       <c r="G190" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="H190" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="I190" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J190" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K190" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="L190" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="M190" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="N190" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
     </row>
     <row r="191" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B191" s="1" t="s">
         <v>15</v>
@@ -8435,33 +8442,33 @@
         <v>18</v>
       </c>
       <c r="G191" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="H191" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="I191" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="J191" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K191" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="L191" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="M191" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="N191" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="192" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B192" s="1" t="s">
         <v>15</v>
@@ -8476,28 +8483,69 @@
         <v>23</v>
       </c>
       <c r="G192" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="H192" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="I192" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="J192" s="1" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="K192" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="L192" s="1" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="M192" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="N192" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
+      </c>
+    </row>
+    <row r="193" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A193" s="3">
+        <v>46029</v>
+      </c>
+      <c r="B193" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C193" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D193" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E193" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="G193" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="H193" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="I193" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="J193" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="K193" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="L193" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="M193" t="s">
+        <v>400</v>
+      </c>
+      <c r="N193" s="2" t="s">
+        <v>400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>